<commit_message>
test: update parser test mode to batch search only
- Modified parser testing to run exclusively in batch search mode
- Removed other test modes to simplify and standardize testing workflow
- Ensured consistency and reliability in parser evaluation process
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/parser_outputs/parsed_result_test_transaction_1.xlsx
+++ b/Text2SQL_Template/output/parser_outputs/parsed_result_test_transaction_1.xlsx
@@ -82,7 +82,7 @@
     <t>SELECT * FROM transaction WHERE reference_id = '5566778899'</t>
   </si>
   <si>
-    <t>SELECT * FROM transaction WHERE reference_id = '3344556677'</t>
+    <t>SELECT * FROM customer WHERE id = '3344556677'</t>
   </si>
   <si>
     <t>SELECT * FROM transaction WHERE reference_id = '9988776655'</t>
@@ -97,7 +97,7 @@
     <t>SELECT * FROM transaction WHERE reference_id = '4455667788'</t>
   </si>
   <si>
-    <t>SELECT * FROM transaction WHERE reference_id = '8899001122'</t>
+    <t>SELECT * FROM customer WHERE id = '8899001122'</t>
   </si>
   <si>
     <t>LOOKUP</t>
@@ -133,7 +133,7 @@
     <t>Tra cứu reference_id = 5566778899</t>
   </si>
   <si>
-    <t>Tra cứu reference_id = 3344556677</t>
+    <t>Tra cứu id = 3344556677</t>
   </si>
   <si>
     <t>Tra cứu reference_id = 9988776655</t>
@@ -148,7 +148,7 @@
     <t>Tra cứu reference_id = 4455667788</t>
   </si>
   <si>
-    <t>Tra cứu reference_id = 8899001122</t>
+    <t>Tra cứu id = 8899001122</t>
   </si>
   <si>
     <t>Không xác định được cột</t>

</xml_diff>